<commit_message>
student insert and sort
</commit_message>
<xml_diff>
--- a/public/Student_Demo_Data.xlsx
+++ b/public/Student_Demo_Data.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Next js\Faculty dashboard\client\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88352E1-66BC-42B6-B71C-0257319115C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9321BEED-5F33-420B-BA1E-ED8498BCCED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Students Demo Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="82">
   <si>
     <t>Student Name</t>
   </si>
@@ -52,9 +65,6 @@
     <t>9876543210</t>
   </si>
   <si>
-    <t>DATA SCIENCE</t>
-  </si>
-  <si>
     <t>6 months</t>
   </si>
   <si>
@@ -73,9 +83,6 @@
     <t>9123456780</t>
   </si>
   <si>
-    <t>TALLY PRIME</t>
-  </si>
-  <si>
     <t>3 months</t>
   </si>
   <si>
@@ -94,9 +101,6 @@
     <t>9988776655</t>
   </si>
   <si>
-    <t>CYBER SECURITY &amp; ETHICAL HACKING</t>
-  </si>
-  <si>
     <t>8 months</t>
   </si>
   <si>
@@ -115,18 +119,12 @@
     <t>9012345678</t>
   </si>
   <si>
-    <t>ENGLISH SPEAKING COURSE</t>
-  </si>
-  <si>
     <t>4 months</t>
   </si>
   <si>
     <t>10-02-2026</t>
   </si>
   <si>
-    <t>10:30-12:30</t>
-  </si>
-  <si>
     <t>Weekend</t>
   </si>
   <si>
@@ -136,9 +134,6 @@
     <t>9098765432</t>
   </si>
   <si>
-    <t>MOBILE APPLICATION DEVELOPMENT</t>
-  </si>
-  <si>
     <t>5 months</t>
   </si>
   <si>
@@ -149,16 +144,174 @@
   </si>
   <si>
     <t>rollno</t>
+  </si>
+  <si>
+    <t>10:30-12:00</t>
+  </si>
+  <si>
+    <t>12:00-1:30</t>
+  </si>
+  <si>
+    <t>3:30-5:00</t>
+  </si>
+  <si>
+    <t>English Speaking Course</t>
+  </si>
+  <si>
+    <t>05-01-2027</t>
+  </si>
+  <si>
+    <t>05-01-2028</t>
+  </si>
+  <si>
+    <t>05-01-2029</t>
+  </si>
+  <si>
+    <t>05-01-2030</t>
+  </si>
+  <si>
+    <t>05-01-2031</t>
+  </si>
+  <si>
+    <t>05-01-2032</t>
+  </si>
+  <si>
+    <t>05-01-2033</t>
+  </si>
+  <si>
+    <t>05-01-2034</t>
+  </si>
+  <si>
+    <t>05-01-2035</t>
+  </si>
+  <si>
+    <t>05-01-2036</t>
+  </si>
+  <si>
+    <t>05-01-2037</t>
+  </si>
+  <si>
+    <t>05-01-2038</t>
+  </si>
+  <si>
+    <t>05-01-2039</t>
+  </si>
+  <si>
+    <t>05-01-2040</t>
+  </si>
+  <si>
+    <t>05-01-2041</t>
+  </si>
+  <si>
+    <t>05-01-2042</t>
+  </si>
+  <si>
+    <t>  DCAP</t>
+  </si>
+  <si>
+    <t>  ADCE</t>
+  </si>
+  <si>
+    <t>  AI&amp;ML</t>
+  </si>
+  <si>
+    <t>  MDCE</t>
+  </si>
+  <si>
+    <t>  PDSHE</t>
+  </si>
+  <si>
+    <t>  SOFTWARE&amp;HARDWARE</t>
+  </si>
+  <si>
+    <t>  PDSEA</t>
+  </si>
+  <si>
+    <t>  DCHN</t>
+  </si>
+  <si>
+    <t>  ADCHN</t>
+  </si>
+  <si>
+    <t>  E-ACCOUNTING</t>
+  </si>
+  <si>
+    <t>  TALLY PRIME</t>
+  </si>
+  <si>
+    <t>  PDEA</t>
+  </si>
+  <si>
+    <t>  ADEA</t>
+  </si>
+  <si>
+    <t>  ANIMATION</t>
+  </si>
+  <si>
+    <t>  ADVANCE ANIMATION</t>
+  </si>
+  <si>
+    <t>  MASTERS IN ANIMATION</t>
+  </si>
+  <si>
+    <t>  DIPLOMA IN WEBSITE ENGINEERING</t>
+  </si>
+  <si>
+    <t>  ADVANCE DIPLOMA IN WEBSITE ENGINEERING</t>
+  </si>
+  <si>
+    <t>  DM</t>
+  </si>
+  <si>
+    <t>  CYBER SECURITY &amp; ETHICAL HACKING</t>
+  </si>
+  <si>
+    <t>  DATA SCIENCE</t>
+  </si>
+  <si>
+    <t>  CHATGPT</t>
+  </si>
+  <si>
+    <t>  MOBILE APPLICATION DEVELOPMENT</t>
+  </si>
+  <si>
+    <t>  CLOUD COMPUTING</t>
+  </si>
+  <si>
+    <t>  BPO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -184,8 +337,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,18 +650,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="47.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -507,7 +671,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -528,7 +692,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -538,142 +702,786 @@
       <c r="C2">
         <v>2457</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2">
+        <v>1152</v>
+      </c>
+      <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="F2">
-        <v>5500</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>12</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>13</v>
       </c>
-      <c r="I2" t="s">
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
       </c>
       <c r="C3">
         <v>2469</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3">
+        <v>1029</v>
+      </c>
+      <c r="G3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
         <v>18</v>
       </c>
-      <c r="F3">
-        <v>4000</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>19</v>
       </c>
-      <c r="H3" t="s">
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>20</v>
       </c>
-      <c r="I3" t="s">
+      <c r="B4" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
       </c>
       <c r="C4">
         <v>2347</v>
       </c>
-      <c r="D4" t="s">
-        <v>24</v>
+      <c r="D4" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4">
+        <v>1548</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" t="s">
         <v>25</v>
       </c>
-      <c r="F4">
-        <v>7000</v>
-      </c>
-      <c r="G4" t="s">
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>26</v>
       </c>
-      <c r="H4" t="s">
+      <c r="B5" t="s">
         <v>27</v>
-      </c>
-      <c r="I4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
       </c>
       <c r="C5">
         <v>2258</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5">
+        <v>1410</v>
+      </c>
+      <c r="G5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>31</v>
       </c>
-      <c r="E5" t="s">
+      <c r="B6" t="s">
         <v>32</v>
-      </c>
-      <c r="F5">
-        <v>3000</v>
-      </c>
-      <c r="G5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" t="s">
-        <v>37</v>
       </c>
       <c r="C6">
         <v>2687</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6">
+        <v>967</v>
+      </c>
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" t="s">
+        <v>13</v>
+      </c>
+      <c r="N6" s="1"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>2457</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7">
+        <v>1407</v>
+      </c>
+      <c r="G7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>13</v>
+      </c>
+      <c r="N7" s="2"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>2469</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8">
+        <v>1678</v>
+      </c>
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I8" t="s">
+        <v>19</v>
+      </c>
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9">
+        <v>2347</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9">
+        <v>1482</v>
+      </c>
+      <c r="G9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" t="s">
+        <v>37</v>
+      </c>
+      <c r="I9" t="s">
+        <v>25</v>
+      </c>
+      <c r="N9" s="2"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>2258</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10">
+        <v>1308</v>
+      </c>
+      <c r="G10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" t="s">
         <v>38</v>
       </c>
-      <c r="E6" t="s">
+      <c r="I10" t="s">
+        <v>30</v>
+      </c>
+      <c r="N10" s="2"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11">
+        <v>2687</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11">
+        <v>1493</v>
+      </c>
+      <c r="G11" t="s">
+        <v>34</v>
+      </c>
+      <c r="H11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11" t="s">
+        <v>13</v>
+      </c>
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12">
+        <v>2458</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12">
+        <v>1604</v>
+      </c>
+      <c r="G12" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" t="s">
+        <v>13</v>
+      </c>
+      <c r="N12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13">
+        <v>2457</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13">
+        <v>1746</v>
+      </c>
+      <c r="G13" t="s">
+        <v>42</v>
+      </c>
+      <c r="H13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I13" t="s">
+        <v>19</v>
+      </c>
+      <c r="N13" s="2"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14">
+        <v>2469</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14">
+        <v>1159</v>
+      </c>
+      <c r="G14" t="s">
+        <v>43</v>
+      </c>
+      <c r="H14" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" t="s">
+        <v>25</v>
+      </c>
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15">
+        <v>2347</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15">
+        <v>1527</v>
+      </c>
+      <c r="G15" t="s">
+        <v>44</v>
+      </c>
+      <c r="H15" t="s">
+        <v>38</v>
+      </c>
+      <c r="I15" t="s">
+        <v>30</v>
+      </c>
+      <c r="N15" s="2"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16">
+        <v>2258</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16">
+        <v>1142</v>
+      </c>
+      <c r="G16" t="s">
+        <v>45</v>
+      </c>
+      <c r="H16" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" t="s">
+        <v>13</v>
+      </c>
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17">
+        <v>2687</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17">
+        <v>1714</v>
+      </c>
+      <c r="G17" t="s">
+        <v>46</v>
+      </c>
+      <c r="H17" t="s">
         <v>39</v>
       </c>
-      <c r="F6">
-        <v>6000</v>
-      </c>
-      <c r="G6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="I17" t="s">
+        <v>13</v>
+      </c>
+      <c r="N17" s="2"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18">
+        <v>2457</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18">
+        <v>1573</v>
+      </c>
+      <c r="G18" t="s">
+        <v>47</v>
+      </c>
+      <c r="H18" t="s">
+        <v>24</v>
+      </c>
+      <c r="I18" t="s">
+        <v>19</v>
+      </c>
+      <c r="N18" s="2"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19">
+        <v>2469</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19" t="s">
+        <v>22</v>
+      </c>
+      <c r="F19">
+        <v>1601</v>
+      </c>
+      <c r="G19" t="s">
+        <v>48</v>
+      </c>
+      <c r="H19" t="s">
+        <v>37</v>
+      </c>
+      <c r="I19" t="s">
+        <v>25</v>
+      </c>
+      <c r="N19" s="2"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20">
+        <v>2347</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20">
+        <v>1193</v>
+      </c>
+      <c r="G20" t="s">
+        <v>49</v>
+      </c>
+      <c r="H20" t="s">
+        <v>38</v>
+      </c>
+      <c r="I20" t="s">
+        <v>30</v>
+      </c>
+      <c r="N20" s="2"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21">
+        <v>2258</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E21" t="s">
+        <v>33</v>
+      </c>
+      <c r="F21">
+        <v>1529</v>
+      </c>
+      <c r="G21" t="s">
+        <v>50</v>
+      </c>
+      <c r="H21" t="s">
+        <v>35</v>
+      </c>
+      <c r="I21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N21" s="2"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>14</v>
       </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22">
+        <v>2687</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E22" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22">
+        <v>1091</v>
+      </c>
+      <c r="G22" t="s">
+        <v>51</v>
+      </c>
+      <c r="H22" t="s">
+        <v>12</v>
+      </c>
+      <c r="I22" t="s">
+        <v>13</v>
+      </c>
+      <c r="N22" s="2"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23">
+        <v>2458</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E23" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23">
+        <v>1640</v>
+      </c>
+      <c r="G23" t="s">
+        <v>52</v>
+      </c>
+      <c r="H23" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" t="s">
+        <v>19</v>
+      </c>
+      <c r="N23" s="2"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24">
+        <v>2457</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24">
+        <v>1298</v>
+      </c>
+      <c r="G24" t="s">
+        <v>53</v>
+      </c>
+      <c r="H24" t="s">
+        <v>37</v>
+      </c>
+      <c r="I24" t="s">
+        <v>25</v>
+      </c>
+      <c r="N24" s="2"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25">
+        <v>2469</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E25" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25">
+        <v>1319</v>
+      </c>
+      <c r="G25" t="s">
+        <v>54</v>
+      </c>
+      <c r="H25" t="s">
+        <v>38</v>
+      </c>
+      <c r="I25" t="s">
+        <v>30</v>
+      </c>
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26">
+        <v>2347</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26">
+        <v>1469</v>
+      </c>
+      <c r="G26" t="s">
+        <v>55</v>
+      </c>
+      <c r="H26" t="s">
+        <v>35</v>
+      </c>
+      <c r="I26" t="s">
+        <v>13</v>
+      </c>
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27">
+        <v>2258</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" t="s">
+        <v>10</v>
+      </c>
+      <c r="F27">
+        <v>1449</v>
+      </c>
+      <c r="G27" t="s">
+        <v>56</v>
+      </c>
+      <c r="H27" t="s">
+        <v>39</v>
+      </c>
+      <c r="I27" t="s">
+        <v>13</v>
+      </c>
+      <c r="N27" s="2"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N28" s="2"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N29" s="2"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N30" s="2"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N31" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>